<commit_message>
Libreta de tareas única, aviso de examen de colocación, plazo de 7 días solo para efectivo y Excel con el formato del colegio
</commit_message>
<xml_diff>
--- a/listas/Cambios en las listas 2026-2027.xlsx
+++ b/listas/Cambios en las listas 2026-2027.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E276"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -655,7 +655,7 @@
         <v>210</v>
       </c>
       <c r="D15" t="str">
-        <v>Libreta de tareas Liceo Alexander Dul</v>
+        <v>Libreta de tareas</v>
       </c>
       <c r="E15">
         <v>210</v>
@@ -893,7 +893,7 @@
         <v>210</v>
       </c>
       <c r="D29" t="str">
-        <v>Libreta de tareas Liceo Alexander Dul</v>
+        <v>Libreta de tareas</v>
       </c>
       <c r="E29">
         <v>210</v>
@@ -1148,7 +1148,7 @@
         <v>210</v>
       </c>
       <c r="D44" t="str">
-        <v>Libreta de tareas Liceo Alexander Dul</v>
+        <v>Libreta de tareas</v>
       </c>
       <c r="E44">
         <v>210</v>
@@ -1505,7 +1505,7 @@
         <v>210</v>
       </c>
       <c r="D65" t="str">
-        <v>Libreta de tareas Liceo Alexander Dul</v>
+        <v>Libreta de tareas</v>
       </c>
       <c r="E65">
         <v>210</v>
@@ -1828,7 +1828,7 @@
         <v>210</v>
       </c>
       <c r="D84" t="str">
-        <v>Libreta de tareas Liceo Alexander Dul</v>
+        <v>Libreta de tareas</v>
       </c>
       <c r="E84">
         <v>210</v>
@@ -2151,7 +2151,7 @@
         <v>210</v>
       </c>
       <c r="D103" t="str">
-        <v>Libreta de tareas Liceo Alexander Dul</v>
+        <v>Libreta de tareas</v>
       </c>
       <c r="E103">
         <v>210</v>
@@ -2400,16 +2400,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B118" t="str">
-        <v>Libreta de tareas</v>
+        <v>Lápiz adhesivo tipo pritt 220 grs</v>
       </c>
       <c r="C118">
-        <v>210</v>
+        <v>40</v>
       </c>
       <c r="D118" t="str">
-        <v>Libreta de tareas Colegio Floresta</v>
+        <v>Lápiz adhesivo tipo Pritt 22 g</v>
       </c>
       <c r="E118">
-        <v>210</v>
+        <v>40</v>
       </c>
     </row>
     <row r="119">
@@ -2417,16 +2417,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B119" t="str">
-        <v>Lápiz adhesivo tipo pritt 220 grs</v>
+        <v>Block papel albanene</v>
       </c>
       <c r="C119">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="D119" t="str">
-        <v>Lápiz adhesivo tipo Pritt 22 g</v>
+        <v>Block de papel albanene</v>
       </c>
       <c r="E119">
-        <v>40</v>
+        <v>90</v>
       </c>
     </row>
     <row r="120">
@@ -2434,16 +2434,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B120" t="str">
-        <v>Block papel albanene</v>
+        <v>Plumas de tinta rosa</v>
       </c>
       <c r="C120">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="D120" t="str">
-        <v>Block de papel albanene</v>
+        <v>Bolígrafo de tinta rosa</v>
       </c>
       <c r="E120">
-        <v>90</v>
+        <v>10</v>
       </c>
     </row>
     <row r="121">
@@ -2451,13 +2451,13 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B121" t="str">
-        <v>Plumas de tinta rosa</v>
+        <v>Plumas de tinta negra</v>
       </c>
       <c r="C121">
         <v>10</v>
       </c>
       <c r="D121" t="str">
-        <v>Bolígrafo de tinta rosa</v>
+        <v>Bolígrafo de tinta negra</v>
       </c>
       <c r="E121">
         <v>10</v>
@@ -2468,16 +2468,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B122" t="str">
-        <v>Plumas de tinta negra</v>
-      </c>
-      <c r="C122">
-        <v>10</v>
+        <v>(repetido) Plumas de tinta negra</v>
+      </c>
+      <c r="C122" t="str">
+        <v>cant. 3</v>
       </c>
       <c r="D122" t="str">
-        <v>Bolígrafo de tinta negra</v>
-      </c>
-      <c r="E122">
-        <v>10</v>
+        <v>sumado a Bolígrafo de tinta negra</v>
+      </c>
+      <c r="E122" t="str">
+        <v>cant. 4</v>
       </c>
     </row>
     <row r="123">
@@ -2485,16 +2485,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B123" t="str">
-        <v>(repetido) Plumas de tinta negra</v>
-      </c>
-      <c r="C123" t="str">
-        <v>cant. 3</v>
+        <v>Plumas de tinta azul</v>
+      </c>
+      <c r="C123">
+        <v>10</v>
       </c>
       <c r="D123" t="str">
-        <v>sumado a Bolígrafo de tinta negra</v>
-      </c>
-      <c r="E123" t="str">
-        <v>cant. 4</v>
+        <v>Bolígrafo de tinta azul</v>
+      </c>
+      <c r="E123">
+        <v>10</v>
       </c>
     </row>
     <row r="124">
@@ -2502,16 +2502,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B124" t="str">
-        <v>Plumas de tinta azul</v>
-      </c>
-      <c r="C124">
-        <v>10</v>
+        <v>(repetido) Plumas de tinta azul</v>
+      </c>
+      <c r="C124" t="str">
+        <v>cant. 2</v>
       </c>
       <c r="D124" t="str">
-        <v>Bolígrafo de tinta azul</v>
-      </c>
-      <c r="E124">
-        <v>10</v>
+        <v>sumado a Bolígrafo de tinta azul</v>
+      </c>
+      <c r="E124" t="str">
+        <v>cant. 3</v>
       </c>
     </row>
     <row r="125">
@@ -2519,16 +2519,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B125" t="str">
-        <v>(repetido) Plumas de tinta azul</v>
-      </c>
-      <c r="C125" t="str">
-        <v>cant. 2</v>
+        <v>Plumón para pizarrón blanco magistral (negro, azul, rojo y verde)</v>
+      </c>
+      <c r="C125">
+        <v>35</v>
       </c>
       <c r="D125" t="str">
-        <v>sumado a Bolígrafo de tinta azul</v>
-      </c>
-      <c r="E125" t="str">
-        <v>cant. 3</v>
+        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
+      </c>
+      <c r="E125">
+        <v>35</v>
       </c>
     </row>
     <row r="126">
@@ -2536,16 +2536,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B126" t="str">
-        <v>Plumón para pizarrón blanco magistral (negro, azul, rojo y verde)</v>
+        <v>Lápiz adhesivo 42gr</v>
       </c>
       <c r="C126">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="D126" t="str">
-        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
+        <v>Lápiz adhesivo tipo Pritt 42 g</v>
       </c>
       <c r="E126">
-        <v>35</v>
+        <v>75</v>
       </c>
     </row>
     <row r="127">
@@ -2553,16 +2553,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B127" t="str">
-        <v>Lápiz adhesivo 42gr</v>
+        <v>Paquete de 300 hojas blancas</v>
       </c>
       <c r="C127">
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="D127" t="str">
-        <v>Lápiz adhesivo tipo Pritt 42 g</v>
+        <v>Paquete de 300 hojas blancas tamaño carta</v>
       </c>
       <c r="E127">
-        <v>75</v>
+        <v>135</v>
       </c>
     </row>
     <row r="128">
@@ -2570,16 +2570,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B128" t="str">
-        <v>Paquete de 300 hojas blancas</v>
+        <v>Bote de pintura vinci cualquier color</v>
       </c>
       <c r="C128">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="D128" t="str">
-        <v>Paquete de 300 hojas blancas tamaño carta</v>
+        <v>Bote de pintura Vinci · Cualquier color</v>
       </c>
       <c r="E128">
-        <v>135</v>
+        <v>25</v>
       </c>
     </row>
     <row r="129">
@@ -2587,16 +2587,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B129" t="str">
-        <v>Bote de pintura vinci cualquier color</v>
+        <v>Cartulinas blancas</v>
       </c>
       <c r="C129">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D129" t="str">
-        <v>Bote de pintura Vinci · Cualquier color</v>
+        <v>Cartulina blanca</v>
       </c>
       <c r="E129">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="130">
@@ -2604,16 +2604,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B130" t="str">
-        <v>Cartulinas blancas</v>
+        <v>Pliegos de mica</v>
       </c>
       <c r="C130">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D130" t="str">
-        <v>Cartulina blanca</v>
+        <v>Pliego de mica</v>
       </c>
       <c r="E130">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="131">
@@ -2621,16 +2621,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B131" t="str">
-        <v>Pliegos de mica</v>
+        <v>Hojas de foami</v>
       </c>
       <c r="C131">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="D131" t="str">
-        <v>Pliego de mica</v>
+        <v>Hoja de foami tamaño carta · Diferentes colores</v>
       </c>
       <c r="E131">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="132">
@@ -2638,16 +2638,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B132" t="str">
-        <v>Hojas de foami</v>
+        <v>Hojas de foami diamantado</v>
       </c>
       <c r="C132">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D132" t="str">
-        <v>Hoja de foami tamaño carta · Diferentes colores</v>
+        <v>Hoja de foami diamantado</v>
       </c>
       <c r="E132">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="133">
@@ -2655,16 +2655,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B133" t="str">
-        <v>Hojas de foami diamantado</v>
+        <v>Marca textos</v>
       </c>
       <c r="C133">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D133" t="str">
-        <v>Hoja de foami diamantado</v>
+        <v>Marcatextos</v>
       </c>
       <c r="E133">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="134">
@@ -2672,16 +2672,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B134" t="str">
-        <v>Marca textos</v>
+        <v>Jabón líquido para manos</v>
       </c>
       <c r="C134">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="D134" t="str">
-        <v>Marcatextos</v>
+        <v>Jabón líquido para manos 225 ml</v>
       </c>
       <c r="E134">
-        <v>35</v>
+        <v>60</v>
       </c>
     </row>
     <row r="135">
@@ -2689,16 +2689,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B135" t="str">
-        <v>Jabón líquido para manos</v>
+        <v>Sobre amarillos tamaño carta</v>
       </c>
       <c r="C135">
-        <v>60</v>
+        <v>9</v>
       </c>
       <c r="D135" t="str">
-        <v>Jabón líquido para manos 225 ml</v>
+        <v>Sobre amarillo tamaño carta</v>
       </c>
       <c r="E135">
-        <v>60</v>
+        <v>9</v>
       </c>
     </row>
     <row r="136">
@@ -2706,16 +2706,16 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B136" t="str">
-        <v>Sobre amarillos tamaño carta</v>
+        <v>Gateway to the world A1+ Student´s book (Básico) ISBN: 9781380042309</v>
       </c>
       <c r="C136">
-        <v>9</v>
+        <v>1145</v>
       </c>
       <c r="D136" t="str">
-        <v>Sobre amarillo tamaño carta</v>
+        <v>Gateway to the World A1+ Student's book ISBN: 9781380042309</v>
       </c>
       <c r="E136">
-        <v>9</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="137">
@@ -2723,13 +2723,13 @@
         <v>1ro SECUNDARIA</v>
       </c>
       <c r="B137" t="str">
-        <v>Gateway to the world A1+ Student´s book (Básico) ISBN: 9781380042309</v>
+        <v>Gateway to the world A2 Student´s book (Avanzado) ISBN: 9781380042507</v>
       </c>
       <c r="C137">
         <v>1145</v>
       </c>
       <c r="D137" t="str">
-        <v>Gateway to the World A1+ Student's book ISBN: 9781380042309</v>
+        <v>Gateway to the World A2 Student's book ISBN: 9781380042507</v>
       </c>
       <c r="E137">
         <v>1145</v>
@@ -2737,19 +2737,19 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>1ro SECUNDARIA</v>
+        <v>2do SECUNDARIA</v>
       </c>
       <c r="B138" t="str">
-        <v>Gateway to the world A2 Student´s book (Avanzado) ISBN: 9781380042507</v>
+        <v>Cuaderno profesional 100hojas CUADRO CHICO (Frances,educación física (comparten), innovación, socioemocional (comparten) e Historia)</v>
       </c>
       <c r="C138">
-        <v>1145</v>
+        <v>150</v>
       </c>
       <c r="D138" t="str">
-        <v>Gateway to the World A2 Student's book ISBN: 9781380042507</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Francés, educación física (comparten), innovación, socioemocional (comparten) e Historia</v>
       </c>
       <c r="E138">
-        <v>1145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="139">
@@ -2757,13 +2757,13 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B139" t="str">
-        <v>Cuaderno profesional 100hojas CUADRO CHICO (Frances,educación física (comparten), innovación, socioemocional (comparten) e Historia)</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas (inglés)</v>
       </c>
       <c r="C139">
         <v>150</v>
       </c>
       <c r="D139" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Francés, educación física (comparten), innovación, socioemocional (comparten) e Historia</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Inglés</v>
       </c>
       <c r="E139">
         <v>150</v>
@@ -2774,13 +2774,13 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B140" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas (inglés)</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas (español)</v>
       </c>
       <c r="C140">
         <v>150</v>
       </c>
       <c r="D140" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Inglés</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Español</v>
       </c>
       <c r="E140">
         <v>150</v>
@@ -2791,13 +2791,13 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B141" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas (español)</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas (matemáticas)</v>
       </c>
       <c r="C141">
         <v>150</v>
       </c>
       <c r="D141" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Español</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
       </c>
       <c r="E141">
         <v>150</v>
@@ -2808,16 +2808,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B142" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas (matemáticas)</v>
+        <v>Constitución Política de México (Educación Cívica)</v>
       </c>
       <c r="C142">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="D142" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
+        <v>Constitución Política de los Estados Unidos Mexicanos</v>
       </c>
       <c r="E142">
-        <v>150</v>
+        <v>100</v>
       </c>
     </row>
     <row r="143">
@@ -2825,16 +2825,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B143" t="str">
-        <v>Constitución Política de México (Educación Cívica)</v>
+        <v>Lápiz adhesivo tipo pritt 22 grs</v>
       </c>
       <c r="C143">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="D143" t="str">
-        <v>Constitución Política de los Estados Unidos Mexicanos</v>
+        <v>Lápiz adhesivo tipo Pritt 22 g</v>
       </c>
       <c r="E143">
-        <v>100</v>
+        <v>40</v>
       </c>
     </row>
     <row r="144">
@@ -2842,16 +2842,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B144" t="str">
-        <v>Lápiz adhesivo tipo pritt 22 grs</v>
+        <v>Lápiz</v>
       </c>
       <c r="C144">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D144" t="str">
-        <v>Lápiz adhesivo tipo Pritt 22 g</v>
+        <v>Lápiz No. 2</v>
       </c>
       <c r="E144">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="145">
@@ -2859,16 +2859,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B145" t="str">
-        <v>Lápiz</v>
+        <v>Tijeras punta roma</v>
       </c>
       <c r="C145">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D145" t="str">
-        <v>Lápiz No. 2</v>
+        <v>Tijeras de punta roma</v>
       </c>
       <c r="E145">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="146">
@@ -2876,16 +2876,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B146" t="str">
-        <v>Tijeras punta roma</v>
+        <v>Goma</v>
       </c>
       <c r="C146">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D146" t="str">
-        <v>Tijeras de punta roma</v>
+        <v>Goma de migajón</v>
       </c>
       <c r="E146">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="147">
@@ -2893,16 +2893,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B147" t="str">
-        <v>Goma</v>
+        <v>Sacapuntas</v>
       </c>
       <c r="C147">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D147" t="str">
-        <v>Goma de migajón</v>
+        <v>Sacapuntas con depósito</v>
       </c>
       <c r="E147">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="148">
@@ -2910,16 +2910,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B148" t="str">
-        <v>Sacapuntas</v>
+        <v>Plumas de tinta negra</v>
       </c>
       <c r="C148">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D148" t="str">
-        <v>Sacapuntas con depósito</v>
+        <v>Bolígrafo de tinta negra</v>
       </c>
       <c r="E148">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="149">
@@ -2927,13 +2927,13 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B149" t="str">
-        <v>Plumas de tinta negra</v>
+        <v>Plumas de tinta azul</v>
       </c>
       <c r="C149">
         <v>10</v>
       </c>
       <c r="D149" t="str">
-        <v>Bolígrafo de tinta negra</v>
+        <v>Bolígrafo de tinta azul</v>
       </c>
       <c r="E149">
         <v>10</v>
@@ -2944,16 +2944,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B150" t="str">
-        <v>Plumas de tinta azul</v>
+        <v>Marca texto (cualquier color)</v>
       </c>
       <c r="C150">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D150" t="str">
-        <v>Bolígrafo de tinta azul</v>
+        <v>Marcatextos</v>
       </c>
       <c r="E150">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="151">
@@ -2961,16 +2961,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B151" t="str">
-        <v>Marca texto (cualquier color)</v>
+        <v>Pluma de tinta roja</v>
       </c>
       <c r="C151">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D151" t="str">
-        <v>Marcatextos</v>
+        <v>Bolígrafo de tinta roja</v>
       </c>
       <c r="E151">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="152">
@@ -2978,16 +2978,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B152" t="str">
-        <v>Pluma de tinta roja</v>
+        <v>Cartulinas de color (diferentes colores)</v>
       </c>
       <c r="C152">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D152" t="str">
-        <v>Bolígrafo de tinta roja</v>
+        <v>Cartulina de color · Diferentes colores</v>
       </c>
       <c r="E152">
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
     <row r="153">
@@ -2995,16 +2995,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B153" t="str">
-        <v>Libreta de tareas</v>
+        <v>Plumón para pizarrón blanco magistral</v>
       </c>
       <c r="C153">
-        <v>210</v>
+        <v>35</v>
       </c>
       <c r="D153" t="str">
-        <v>Libreta de tareas Colegio Floresta</v>
+        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
       </c>
       <c r="E153">
-        <v>210</v>
+        <v>35</v>
       </c>
     </row>
     <row r="154">
@@ -3012,16 +3012,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B154" t="str">
-        <v>Cartulinas de color (diferentes colores)</v>
+        <v>Plumas tinta rosa</v>
       </c>
       <c r="C154">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D154" t="str">
-        <v>Cartulina de color · Diferentes colores</v>
+        <v>Bolígrafo de tinta rosa</v>
       </c>
       <c r="E154">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155">
@@ -3029,16 +3029,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B155" t="str">
-        <v>Plumón para pizarrón blanco magistral</v>
+        <v>Plumas de tinta azul</v>
       </c>
       <c r="C155">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D155" t="str">
-        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
+        <v>Bolígrafo de tinta azul</v>
       </c>
       <c r="E155">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="156">
@@ -3046,16 +3046,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B156" t="str">
-        <v>Plumas tinta rosa</v>
+        <v>Masking</v>
       </c>
       <c r="C156">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D156" t="str">
-        <v>Bolígrafo de tinta rosa</v>
+        <v>Cinta masking tape</v>
       </c>
       <c r="E156">
-        <v>10</v>
+        <v>45</v>
       </c>
     </row>
     <row r="157">
@@ -3063,16 +3063,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B157" t="str">
-        <v>Plumas de tinta azul</v>
+        <v>Paquetes de sanitas. (2 para laboratorio)</v>
       </c>
       <c r="C157">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D157" t="str">
-        <v>Bolígrafo de tinta azul</v>
+        <v>Paquete de Sanitas · 2 para laboratorio</v>
       </c>
       <c r="E157">
-        <v>10</v>
+        <v>50</v>
       </c>
     </row>
     <row r="158">
@@ -3080,16 +3080,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B158" t="str">
-        <v>Masking</v>
+        <v>Bote de pintura vinci cualquier color</v>
       </c>
       <c r="C158">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="D158" t="str">
-        <v>Cinta masking tape</v>
+        <v>Bote de pintura Vinci · Cualquier color</v>
       </c>
       <c r="E158">
-        <v>45</v>
+        <v>25</v>
       </c>
     </row>
     <row r="159">
@@ -3097,16 +3097,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B159" t="str">
-        <v>Paquetes de sanitas. (2 para laboratorio)</v>
+        <v>Sobre amarillos tamaño carta</v>
       </c>
       <c r="C159">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="D159" t="str">
-        <v>Paquete de Sanitas · 2 para laboratorio</v>
+        <v>Sobre amarillo tamaño carta</v>
       </c>
       <c r="E159">
-        <v>50</v>
+        <v>9</v>
       </c>
     </row>
     <row r="160">
@@ -3114,16 +3114,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B160" t="str">
-        <v>Bote de pintura vinci cualquier color</v>
+        <v>Jabón líquido para manos</v>
       </c>
       <c r="C160">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="D160" t="str">
-        <v>Bote de pintura Vinci · Cualquier color</v>
+        <v>Jabón líquido para manos 225 ml</v>
       </c>
       <c r="E160">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="161">
@@ -3131,16 +3131,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B161" t="str">
-        <v>Sobre amarillos tamaño carta</v>
+        <v>Folders color beige tamaño carta</v>
       </c>
       <c r="C161">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D161" t="str">
-        <v>Sobre amarillo tamaño carta</v>
+        <v>Fólder tamaño carta beige</v>
       </c>
       <c r="E161">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="162">
@@ -3148,16 +3148,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B162" t="str">
-        <v>Jabón líquido para manos</v>
+        <v>Rollos de papel Kraft</v>
       </c>
       <c r="C162">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="D162" t="str">
-        <v>Jabón líquido para manos 225 ml</v>
+        <v>Rollo de papel kraft</v>
       </c>
       <c r="E162">
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="163">
@@ -3165,16 +3165,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B163" t="str">
-        <v>Folders color beige tamaño carta</v>
+        <v>Silicón líquido</v>
       </c>
       <c r="C163">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="D163" t="str">
-        <v>Fólder tamaño carta beige</v>
+        <v>Silicón frío 100 ml</v>
       </c>
       <c r="E163">
-        <v>7</v>
+        <v>40</v>
       </c>
     </row>
     <row r="164">
@@ -3182,16 +3182,16 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B164" t="str">
-        <v>Rollos de papel Kraft</v>
+        <v>Gateway to the world A2 Student´s book (Básico) ISBN: 9781380042507</v>
       </c>
       <c r="C164">
-        <v>15</v>
+        <v>1145</v>
       </c>
       <c r="D164" t="str">
-        <v>Rollo de papel kraft</v>
+        <v>Gateway to the World A2 Student's book ISBN: 9781380042507</v>
       </c>
       <c r="E164">
-        <v>15</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="165">
@@ -3199,50 +3199,50 @@
         <v>2do SECUNDARIA</v>
       </c>
       <c r="B165" t="str">
-        <v>Silicón líquido</v>
+        <v>Gateway to the world B1 Student´s book (Avanzado) ISBN: 9781380042699</v>
       </c>
       <c r="C165">
-        <v>40</v>
+        <v>1145</v>
       </c>
       <c r="D165" t="str">
-        <v>Silicón frío 100 ml</v>
+        <v>Gateway to the World B1 Student's book ISBN: 9781380042699</v>
       </c>
       <c r="E165">
-        <v>40</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>2do SECUNDARIA</v>
+        <v>3ro SECUNDARIA</v>
       </c>
       <c r="B166" t="str">
-        <v>Gateway to the world A2 Student´s book (Básico) ISBN: 9781380042507</v>
+        <v>Cuaderno profesional 100hojas CUADRO CHICO (Frances,educación física (comparten), innovación, socioemocional (comparten) e Historia)</v>
       </c>
       <c r="C166">
-        <v>1145</v>
+        <v>150</v>
       </c>
       <c r="D166" t="str">
-        <v>Gateway to the World A2 Student's book ISBN: 9781380042507</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Francés, educación física (comparten), innovación, socioemocional (comparten) e Historia</v>
       </c>
       <c r="E166">
-        <v>1145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>2do SECUNDARIA</v>
+        <v>3ro SECUNDARIA</v>
       </c>
       <c r="B167" t="str">
-        <v>Gateway to the world B1 Student´s book (Avanzado) ISBN: 9781380042699</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas (inglés)</v>
       </c>
       <c r="C167">
-        <v>1145</v>
+        <v>150</v>
       </c>
       <c r="D167" t="str">
-        <v>Gateway to the World B1 Student's book ISBN: 9781380042699</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Inglés</v>
       </c>
       <c r="E167">
-        <v>1145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="168">
@@ -3250,13 +3250,13 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B168" t="str">
-        <v>Cuaderno profesional 100hojas CUADRO CHICO (Frances,educación física (comparten), innovación, socioemocional (comparten) e Historia)</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas (español)</v>
       </c>
       <c r="C168">
         <v>150</v>
       </c>
       <c r="D168" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Francés, educación física (comparten), innovación, socioemocional (comparten) e Historia</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Español</v>
       </c>
       <c r="E168">
         <v>150</v>
@@ -3267,13 +3267,13 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B169" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas (inglés)</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas (matemáticas)</v>
       </c>
       <c r="C169">
         <v>150</v>
       </c>
       <c r="D169" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Inglés</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
       </c>
       <c r="E169">
         <v>150</v>
@@ -3284,16 +3284,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B170" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas (español)</v>
+        <v>Cuaderno profesional NORMA (música)</v>
       </c>
       <c r="C170">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="D170" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Español</v>
+        <v>Cuaderno profesional Norma para música</v>
       </c>
       <c r="E170">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="171">
@@ -3301,16 +3301,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B171" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas (matemáticas)</v>
+        <v>Constitución Política de México (Educación Cívica)</v>
       </c>
       <c r="C171">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="D171" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
+        <v>Constitución Política de los Estados Unidos Mexicanos</v>
       </c>
       <c r="E171">
-        <v>150</v>
+        <v>100</v>
       </c>
     </row>
     <row r="172">
@@ -3318,16 +3318,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B172" t="str">
-        <v>Cuaderno profesional NORMA (música)</v>
+        <v>Lápiz</v>
       </c>
       <c r="C172">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="D172" t="str">
-        <v>Cuaderno profesional Norma para música</v>
+        <v>Lápiz No. 2</v>
       </c>
       <c r="E172">
-        <v>120</v>
+        <v>10</v>
       </c>
     </row>
     <row r="173">
@@ -3335,16 +3335,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B173" t="str">
-        <v>Constitución Política de México (Educación Cívica)</v>
+        <v>Pluma de tinta rosa</v>
       </c>
       <c r="C173">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="D173" t="str">
-        <v>Constitución Política de los Estados Unidos Mexicanos</v>
+        <v>Bolígrafo de tinta rosa</v>
       </c>
       <c r="E173">
-        <v>100</v>
+        <v>10</v>
       </c>
     </row>
     <row r="174">
@@ -3352,13 +3352,13 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B174" t="str">
-        <v>Lápiz</v>
+        <v>Pluma de tinta negra</v>
       </c>
       <c r="C174">
         <v>10</v>
       </c>
       <c r="D174" t="str">
-        <v>Lápiz No. 2</v>
+        <v>Bolígrafo de tinta negra</v>
       </c>
       <c r="E174">
         <v>10</v>
@@ -3369,13 +3369,13 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B175" t="str">
-        <v>Pluma de tinta rosa</v>
+        <v>Pluma de tinta azul</v>
       </c>
       <c r="C175">
         <v>10</v>
       </c>
       <c r="D175" t="str">
-        <v>Bolígrafo de tinta rosa</v>
+        <v>Bolígrafo de tinta azul</v>
       </c>
       <c r="E175">
         <v>10</v>
@@ -3386,13 +3386,13 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B176" t="str">
-        <v>Pluma de tinta negra</v>
+        <v>Goma</v>
       </c>
       <c r="C176">
         <v>10</v>
       </c>
       <c r="D176" t="str">
-        <v>Bolígrafo de tinta negra</v>
+        <v>Goma de migajón</v>
       </c>
       <c r="E176">
         <v>10</v>
@@ -3403,16 +3403,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B177" t="str">
-        <v>Pluma de tinta azul</v>
+        <v>Sacapuntas</v>
       </c>
       <c r="C177">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D177" t="str">
-        <v>Bolígrafo de tinta azul</v>
+        <v>Sacapuntas con depósito</v>
       </c>
       <c r="E177">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="178">
@@ -3420,16 +3420,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B178" t="str">
-        <v>Goma</v>
+        <v>Pritt 22 gr</v>
       </c>
       <c r="C178">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D178" t="str">
-        <v>Goma de migajón</v>
+        <v>Lápiz adhesivo tipo Pritt 22 g</v>
       </c>
       <c r="E178">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="179">
@@ -3437,16 +3437,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B179" t="str">
-        <v>Sacapuntas</v>
+        <v>Tijeras punta roma</v>
       </c>
       <c r="C179">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D179" t="str">
-        <v>Sacapuntas con depósito</v>
+        <v>Tijeras de punta roma</v>
       </c>
       <c r="E179">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="180">
@@ -3454,16 +3454,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B180" t="str">
-        <v>Pritt 22 gr</v>
+        <v>Marca texto (cualquier color)</v>
       </c>
       <c r="C180">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D180" t="str">
-        <v>Lápiz adhesivo tipo Pritt 22 g</v>
+        <v>Marcatextos</v>
       </c>
       <c r="E180">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="181">
@@ -3471,16 +3471,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B181" t="str">
-        <v>Tijeras punta roma</v>
+        <v>Tabla periódica Ed. Patria Actualizada</v>
       </c>
       <c r="C181">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D181" t="str">
-        <v>Tijeras de punta roma</v>
+        <v>Tabla periódica actualizada Ed. Patria</v>
       </c>
       <c r="E181">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="182">
@@ -3488,16 +3488,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B182" t="str">
-        <v>Marca texto (cualquier color)</v>
+        <v>Cartulinas de color (diferentes colores)</v>
       </c>
       <c r="C182">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="D182" t="str">
-        <v>Marcatextos</v>
+        <v>Cartulina de color · Diferentes colores</v>
       </c>
       <c r="E182">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="183">
@@ -3505,16 +3505,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B183" t="str">
-        <v>Libreta de tareas</v>
+        <v>Plumón para pizarrón blanco magistral</v>
       </c>
       <c r="C183">
-        <v>210</v>
+        <v>35</v>
       </c>
       <c r="D183" t="str">
-        <v>Libreta de tareas Colegio Floresta</v>
+        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
       </c>
       <c r="E183">
-        <v>210</v>
+        <v>35</v>
       </c>
     </row>
     <row r="184">
@@ -3522,16 +3522,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B184" t="str">
-        <v>Tabla periódica Ed. Patria Actualizada</v>
+        <v>Plumas tinta negra</v>
       </c>
       <c r="C184">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D184" t="str">
-        <v>Tabla periódica actualizada Ed. Patria</v>
+        <v>Bolígrafo de tinta negra</v>
       </c>
       <c r="E184">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="185">
@@ -3539,16 +3539,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B185" t="str">
-        <v>Cartulinas de color (diferentes colores)</v>
+        <v>Plumas de tinta azul</v>
       </c>
       <c r="C185">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D185" t="str">
-        <v>Cartulina de color · Diferentes colores</v>
+        <v>Bolígrafo de tinta azul</v>
       </c>
       <c r="E185">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="186">
@@ -3556,16 +3556,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B186" t="str">
-        <v>Plumón para pizarrón blanco magistral</v>
+        <v>Paquetes de sanitas.(2 para laboratorio)</v>
       </c>
       <c r="C186">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D186" t="str">
-        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
+        <v>Paquete de Sanitas · 2 para laboratorio</v>
       </c>
       <c r="E186">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="187">
@@ -3573,16 +3573,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B187" t="str">
-        <v>Plumas tinta negra</v>
+        <v>Jabón líquido para manos</v>
       </c>
       <c r="C187">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D187" t="str">
-        <v>Bolígrafo de tinta negra</v>
+        <v>Jabón líquido para manos 225 ml</v>
       </c>
       <c r="E187">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="188">
@@ -3590,16 +3590,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B188" t="str">
-        <v>Plumas de tinta azul</v>
+        <v>Folders color beige tamaño carta</v>
       </c>
       <c r="C188">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D188" t="str">
-        <v>Bolígrafo de tinta azul</v>
+        <v>Fólder tamaño carta beige</v>
       </c>
       <c r="E188">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="189">
@@ -3607,16 +3607,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B189" t="str">
-        <v>Paquetes de sanitas.(2 para laboratorio)</v>
+        <v>Diurex grueso</v>
       </c>
       <c r="C189">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="D189" t="str">
-        <v>Paquete de Sanitas · 2 para laboratorio</v>
+        <v>Cinta diurex gruesa</v>
       </c>
       <c r="E189">
-        <v>50</v>
+        <v>65</v>
       </c>
     </row>
     <row r="190">
@@ -3624,16 +3624,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B190" t="str">
-        <v>Jabón líquido para manos</v>
+        <v>Sobre amarillos tamaño carta</v>
       </c>
       <c r="C190">
-        <v>60</v>
+        <v>9</v>
       </c>
       <c r="D190" t="str">
-        <v>Jabón líquido para manos 225 ml</v>
+        <v>Sobre amarillo tamaño carta</v>
       </c>
       <c r="E190">
-        <v>60</v>
+        <v>9</v>
       </c>
     </row>
     <row r="191">
@@ -3641,16 +3641,16 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B191" t="str">
-        <v>Folders color beige tamaño carta</v>
+        <v>Gateway to the world B1 Student´s book (Básico) ISBN: 9781380042699</v>
       </c>
       <c r="C191">
-        <v>7</v>
+        <v>1145</v>
       </c>
       <c r="D191" t="str">
-        <v>Fólder tamaño carta beige</v>
+        <v>Gateway to the World B1 Student's book ISBN: 9781380042699</v>
       </c>
       <c r="E191">
-        <v>7</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="192">
@@ -3658,67 +3658,67 @@
         <v>3ro SECUNDARIA</v>
       </c>
       <c r="B192" t="str">
-        <v>Diurex grueso</v>
+        <v>Gateway to the world B1+ Student´s book (Avanzado) ISBN: 9781380042880</v>
       </c>
       <c r="C192">
-        <v>65</v>
+        <v>1145</v>
       </c>
       <c r="D192" t="str">
-        <v>Cinta diurex gruesa</v>
+        <v>Gateway to the World B1+ Student's book ISBN: 9781380042880</v>
       </c>
       <c r="E192">
-        <v>65</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>3ro SECUNDARIA</v>
+        <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B193" t="str">
-        <v>Sobre amarillos tamaño carta</v>
+        <v>Cuadernos profesional cuadro chico 100 hojas. (Español, Inglés (forro naranja) , Biología, Geografía, Historia).</v>
       </c>
       <c r="C193">
-        <v>9</v>
+        <v>150</v>
       </c>
       <c r="D193" t="str">
-        <v>Sobre amarillo tamaño carta</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Español, Inglés (forro naranja), Biología, Geografía, Historia</v>
       </c>
       <c r="E193">
-        <v>9</v>
+        <v>150</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>3ro SECUNDARIA</v>
+        <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B194" t="str">
-        <v>Gateway to the world B1 Student´s book (Básico) ISBN: 9781380042699</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas (Matemáticas)</v>
       </c>
       <c r="C194">
-        <v>1145</v>
+        <v>150</v>
       </c>
       <c r="D194" t="str">
-        <v>Gateway to the World B1 Student's book ISBN: 9781380042699</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
       </c>
       <c r="E194">
-        <v>1145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>3ro SECUNDARIA</v>
+        <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B195" t="str">
-        <v>Gateway to the world B1+ Student´s book (Avanzado) ISBN: 9781380042880</v>
+        <v>Cuaderno profesional pautado (música)</v>
       </c>
       <c r="C195">
-        <v>1145</v>
+        <v>90</v>
       </c>
       <c r="D195" t="str">
-        <v>Gateway to the World B1+ Student's book ISBN: 9781380042880</v>
+        <v>Cuaderno profesional pautado para música</v>
       </c>
       <c r="E195">
-        <v>1145</v>
+        <v>90</v>
       </c>
     </row>
     <row r="196">
@@ -3726,16 +3726,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B196" t="str">
-        <v>Cuadernos profesional cuadro chico 100 hojas. (Español, Inglés (forro naranja) , Biología, Geografía, Historia).</v>
+        <v>Bata blanca de algodón (con nombre bordado)</v>
       </c>
       <c r="C196">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="D196" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Español, Inglés (forro naranja), Biología, Geografía, Historia</v>
+        <v>Bata blanca de algodón · Con nombre bordado</v>
       </c>
       <c r="E196">
-        <v>150</v>
+        <v>300</v>
       </c>
     </row>
     <row r="197">
@@ -3743,16 +3743,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B197" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas (Matemáticas)</v>
+        <v>Block de hojas milimetricas 50 hojas (Matemáticas)</v>
       </c>
       <c r="C197">
-        <v>150</v>
+        <v>35</v>
       </c>
       <c r="D197" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
+        <v>Block de hojas milimétricas 50 hojas</v>
       </c>
       <c r="E197">
-        <v>150</v>
+        <v>35</v>
       </c>
     </row>
     <row r="198">
@@ -3760,16 +3760,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B198" t="str">
-        <v>Cuaderno profesional pautado (música)</v>
+        <v>Gomas (1 para entregar en la escuela)</v>
       </c>
       <c r="C198">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="D198" t="str">
-        <v>Cuaderno profesional pautado para música</v>
+        <v>Goma de migajón · 1 para entregar en la escuela</v>
       </c>
       <c r="E198">
-        <v>90</v>
+        <v>10</v>
       </c>
     </row>
     <row r="199">
@@ -3777,16 +3777,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B199" t="str">
-        <v>Bata blanca de algodón (con nombre bordado)</v>
+        <v>Lápiz adhesivo (1 para entregar)</v>
       </c>
       <c r="C199">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="D199" t="str">
-        <v>Bata blanca de algodón · Con nombre bordado</v>
+        <v>Lápiz adhesivo tipo Pritt 22 g · 1 para entregar</v>
       </c>
       <c r="E199">
-        <v>300</v>
+        <v>40</v>
       </c>
     </row>
     <row r="200">
@@ -3794,16 +3794,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B200" t="str">
-        <v>Block de hojas milimetricas 50 hojas (Matemáticas)</v>
+        <v>Lápiz Mirado No. 2 (1 se entrega en la escuela)</v>
       </c>
       <c r="C200">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D200" t="str">
-        <v>Block de hojas milimétricas 50 hojas</v>
+        <v>Lápiz No. 2 · 1 se entrega en la escuela</v>
       </c>
       <c r="E200">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="201">
@@ -3811,16 +3811,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B201" t="str">
-        <v>Gomas (1 para entregar en la escuela)</v>
+        <v>Marcatextos de diferentes colores (1 para entregar)</v>
       </c>
       <c r="C201">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D201" t="str">
-        <v>Goma de migajón · 1 para entregar en la escuela</v>
+        <v>Marcatextos · 1 para entregar</v>
       </c>
       <c r="E201">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="202">
@@ -3828,16 +3828,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B202" t="str">
-        <v>Lápiz adhesivo (1 para entregar)</v>
+        <v>Bolígrafo de tinta negra (1 para entregar)</v>
       </c>
       <c r="C202">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D202" t="str">
-        <v>Lápiz adhesivo tipo Pritt 22 g · 1 para entregar</v>
+        <v>Bolígrafo de tinta negra · 1 para entregar</v>
       </c>
       <c r="E202">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="203">
@@ -3845,13 +3845,13 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B203" t="str">
-        <v>Lápiz Mirado No. 2 (1 se entrega en la escuela)</v>
+        <v>Bolígrafo de tinta azul (1 para entregar)</v>
       </c>
       <c r="C203">
         <v>10</v>
       </c>
       <c r="D203" t="str">
-        <v>Lápiz No. 2 · 1 se entrega en la escuela</v>
+        <v>Bolígrafo de tinta azul · 1 para entregar</v>
       </c>
       <c r="E203">
         <v>10</v>
@@ -3862,16 +3862,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B204" t="str">
-        <v>Marcatextos de diferentes colores (1 para entregar)</v>
+        <v>Bolígrafo de tinta verde (1 para entregar)</v>
       </c>
       <c r="C204">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D204" t="str">
-        <v>Marcatextos · 1 para entregar</v>
+        <v>Bolígrafo de tinta verde · 1 para entregar</v>
       </c>
       <c r="E204">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="205">
@@ -3879,13 +3879,13 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B205" t="str">
-        <v>Bolígrafo de tinta negra (1 para entregar)</v>
+        <v>Bolígrafo de tinta roja (1 para entregar)</v>
       </c>
       <c r="C205">
         <v>10</v>
       </c>
       <c r="D205" t="str">
-        <v>Bolígrafo de tinta negra · 1 para entregar</v>
+        <v>Bolígrafo de tinta roja · 1 para entregar</v>
       </c>
       <c r="E205">
         <v>10</v>
@@ -3896,16 +3896,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B206" t="str">
-        <v>Bolígrafo de tinta azul (1 para entregar)</v>
+        <v>Tijeras punta roma</v>
       </c>
       <c r="C206">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D206" t="str">
-        <v>Bolígrafo de tinta azul · 1 para entregar</v>
+        <v>Tijeras de punta roma</v>
       </c>
       <c r="E206">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="207">
@@ -3913,16 +3913,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B207" t="str">
-        <v>Bolígrafo de tinta verde (1 para entregar)</v>
+        <v>Jabón líquido para manos</v>
       </c>
       <c r="C207">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D207" t="str">
-        <v>Bolígrafo de tinta verde · 1 para entregar</v>
+        <v>Jabón líquido para manos 225 ml</v>
       </c>
       <c r="E207">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="208">
@@ -3930,16 +3930,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B208" t="str">
-        <v>Bolígrafo de tinta roja (1 para entregar)</v>
+        <v>Hojas de foami</v>
       </c>
       <c r="C208">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D208" t="str">
-        <v>Bolígrafo de tinta roja · 1 para entregar</v>
+        <v>Hoja de foami tamaño carta · Diferentes colores</v>
       </c>
       <c r="E208">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="209">
@@ -3947,16 +3947,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B209" t="str">
-        <v>Tijeras punta roma</v>
+        <v>Hojas de foami diamantado</v>
       </c>
       <c r="C209">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D209" t="str">
-        <v>Tijeras de punta roma</v>
+        <v>Hoja de foami diamantado</v>
       </c>
       <c r="E209">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="210">
@@ -3964,16 +3964,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B210" t="str">
-        <v>Jabón líquido para manos</v>
+        <v>Paquetes de sanitas</v>
       </c>
       <c r="C210">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D210" t="str">
-        <v>Jabón líquido para manos 225 ml</v>
+        <v>Paquete de Sanitas</v>
       </c>
       <c r="E210">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="211">
@@ -3981,16 +3981,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B211" t="str">
-        <v>Hojas de foami</v>
+        <v>Silicón frío de 100ml</v>
       </c>
       <c r="C211">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="D211" t="str">
-        <v>Hoja de foami tamaño carta · Diferentes colores</v>
+        <v>Silicón frío 100 ml</v>
       </c>
       <c r="E211">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="212">
@@ -3998,16 +3998,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B212" t="str">
-        <v>Hojas de foami diamantado</v>
+        <v>Diurex</v>
       </c>
       <c r="C212">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D212" t="str">
-        <v>Hoja de foami diamantado</v>
+        <v>Cinta diurex</v>
       </c>
       <c r="E212">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="213">
@@ -4015,16 +4015,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B213" t="str">
-        <v>Paquetes de sanitas</v>
+        <v>Masking tape</v>
       </c>
       <c r="C213">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D213" t="str">
-        <v>Paquete de Sanitas</v>
+        <v>Cinta masking tape</v>
       </c>
       <c r="E213">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="214">
@@ -4032,16 +4032,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B214" t="str">
-        <v>Silicón frío de 100ml</v>
+        <v>Paquete de 50 protectores de hojas de carpeta</v>
       </c>
       <c r="C214">
-        <v>40</v>
+        <v>120</v>
       </c>
       <c r="D214" t="str">
-        <v>Silicón frío 100 ml</v>
+        <v>Paquete de 50 protectores de hojas para carpeta</v>
       </c>
       <c r="E214">
-        <v>40</v>
+        <v>120</v>
       </c>
     </row>
     <row r="215">
@@ -4049,16 +4049,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B215" t="str">
-        <v>Diurex</v>
+        <v>Pliegos de papel lustre (color a elegir)</v>
       </c>
       <c r="C215">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D215" t="str">
-        <v>Cinta diurex</v>
+        <v>Pliego de papel lustre · Color a elegir</v>
       </c>
       <c r="E215">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="216">
@@ -4066,16 +4066,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B216" t="str">
-        <v>Masking tape</v>
+        <v>Pliego de papel américa color amarillo</v>
       </c>
       <c r="C216">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D216" t="str">
-        <v>Cinta masking tape</v>
+        <v>Pliego de papel américa amarillo</v>
       </c>
       <c r="E216">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="217">
@@ -4083,16 +4083,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B217" t="str">
-        <v>Paquete de 50 protectores de hojas de carpeta</v>
+        <v>Pliegos de papel Kraft</v>
       </c>
       <c r="C217">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="D217" t="str">
-        <v>Paquete de 50 protectores de hojas para carpeta</v>
+        <v>Pliego de papel kraft</v>
       </c>
       <c r="E217">
-        <v>120</v>
+        <v>15</v>
       </c>
     </row>
     <row r="218">
@@ -4100,16 +4100,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B218" t="str">
-        <v>Pliegos de papel lustre (color a elegir)</v>
+        <v>Plumones para pizarrón blanco, colores: negro, rojo, verde y azul.</v>
       </c>
       <c r="C218">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D218" t="str">
-        <v>Pliego de papel lustre · Color a elegir</v>
+        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
       </c>
       <c r="E218">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="219">
@@ -4117,16 +4117,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B219" t="str">
-        <v>Pliego de papel américa color amarillo</v>
+        <v>Diccionario escolar de la Lengua Española</v>
       </c>
       <c r="C219">
-        <v>30</v>
+        <v>182</v>
       </c>
       <c r="D219" t="str">
-        <v>Pliego de papel américa amarillo</v>
+        <v>Diccionario escolar de la lengua española Larousse</v>
       </c>
       <c r="E219">
-        <v>30</v>
+        <v>182</v>
       </c>
     </row>
     <row r="220">
@@ -4134,16 +4134,16 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B220" t="str">
-        <v>Pliegos de papel Kraft</v>
+        <v>Get Involved! A1+ Student´s book (básico) ISBN: 9781380068750</v>
       </c>
       <c r="C220">
-        <v>15</v>
+        <v>1040</v>
       </c>
       <c r="D220" t="str">
-        <v>Pliego de papel kraft</v>
+        <v>Get Involved! A1+ Student's book ISBN: 9781380068750</v>
       </c>
       <c r="E220">
-        <v>15</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="221">
@@ -4151,67 +4151,67 @@
         <v>1ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B221" t="str">
-        <v>Plumones para pizarrón blanco, colores: negro, rojo, verde y azul.</v>
+        <v>Get Involved! B1 Student´s book (avanzado) ISBN: 9781380068873</v>
       </c>
       <c r="C221">
-        <v>35</v>
+        <v>1040</v>
       </c>
       <c r="D221" t="str">
-        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
+        <v>Get Involved! B1 Student's book ISBN: 9781380068873</v>
       </c>
       <c r="E221">
-        <v>35</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>1ro SECUNDARIA VESPERTINO</v>
+        <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B222" t="str">
-        <v>Diccionario escolar de la Lengua Española</v>
+        <v>Cuadernos profesional cuadro chico 100. (Español, Inglés (forro azul), Física, Historia).</v>
       </c>
       <c r="C222">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="D222" t="str">
-        <v>Diccionario escolar de la lengua española Larousse</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Español, Inglés (forro azul), Física, Historia</v>
       </c>
       <c r="E222">
-        <v>182</v>
+        <v>150</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>1ro SECUNDARIA VESPERTINO</v>
+        <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B223" t="str">
-        <v>Get Involved! A1+ Student´s book (básico) ISBN: 9781380068750</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas Matemáticas</v>
       </c>
       <c r="C223">
-        <v>1040</v>
+        <v>150</v>
       </c>
       <c r="D223" t="str">
-        <v>Get Involved! A1+ Student's book ISBN: 9781380068750</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
       </c>
       <c r="E223">
-        <v>1040</v>
+        <v>150</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>1ro SECUNDARIA VESPERTINO</v>
+        <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B224" t="str">
-        <v>Get Involved! B1 Student´s book (avanzado) ISBN: 9781380068873</v>
+        <v>Bata blanca de algodón (con nombre bordado)</v>
       </c>
       <c r="C224">
-        <v>1040</v>
+        <v>300</v>
       </c>
       <c r="D224" t="str">
-        <v>Get Involved! B1 Student's book ISBN: 9781380068873</v>
+        <v>Bata blanca de algodón · Con nombre bordado</v>
       </c>
       <c r="E224">
-        <v>1040</v>
+        <v>300</v>
       </c>
     </row>
     <row r="225">
@@ -4219,16 +4219,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B225" t="str">
-        <v>Cuadernos profesional cuadro chico 100. (Español, Inglés (forro azul), Física, Historia).</v>
+        <v>Gomas (1 se entrega en la escuela)</v>
       </c>
       <c r="C225">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="D225" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Español, Inglés (forro azul), Física, Historia</v>
+        <v>Goma de migajón · 1 se entrega en la escuela</v>
       </c>
       <c r="E225">
-        <v>150</v>
+        <v>10</v>
       </c>
     </row>
     <row r="226">
@@ -4236,16 +4236,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B226" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas Matemáticas</v>
+        <v>Lápiz adhesivo (1 para entregar)</v>
       </c>
       <c r="C226">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="D226" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
+        <v>Lápiz adhesivo tipo Pritt 22 g · 1 para entregar</v>
       </c>
       <c r="E226">
-        <v>150</v>
+        <v>40</v>
       </c>
     </row>
     <row r="227">
@@ -4253,16 +4253,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B227" t="str">
-        <v>Bata blanca de algodón (con nombre bordado)</v>
+        <v>Lápiz Mirado No. 2 (1 para entregar)</v>
       </c>
       <c r="C227">
-        <v>300</v>
+        <v>10</v>
       </c>
       <c r="D227" t="str">
-        <v>Bata blanca de algodón · Con nombre bordado</v>
+        <v>Lápiz No. 2 · 1 para entregar</v>
       </c>
       <c r="E227">
-        <v>300</v>
+        <v>10</v>
       </c>
     </row>
     <row r="228">
@@ -4270,16 +4270,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B228" t="str">
-        <v>Gomas (1 se entrega en la escuela)</v>
+        <v>Marca texto diferentes colores (1 para entregar)</v>
       </c>
       <c r="C228">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D228" t="str">
-        <v>Goma de migajón · 1 se entrega en la escuela</v>
+        <v>Marcatextos · 1 para entregar</v>
       </c>
       <c r="E228">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="229">
@@ -4287,16 +4287,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B229" t="str">
-        <v>Lápiz adhesivo (1 para entregar)</v>
+        <v>Bolígrafo tinta negra (1 para entregar)</v>
       </c>
       <c r="C229">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D229" t="str">
-        <v>Lápiz adhesivo tipo Pritt 22 g · 1 para entregar</v>
+        <v>Bolígrafo de tinta negra · 1 para entregar</v>
       </c>
       <c r="E229">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230">
@@ -4304,13 +4304,13 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B230" t="str">
-        <v>Lápiz Mirado No. 2 (1 para entregar)</v>
+        <v>Bolígrafo tinta azul (1 para entregar)</v>
       </c>
       <c r="C230">
         <v>10</v>
       </c>
       <c r="D230" t="str">
-        <v>Lápiz No. 2 · 1 para entregar</v>
+        <v>Bolígrafo de tinta azul · 1 para entregar</v>
       </c>
       <c r="E230">
         <v>10</v>
@@ -4321,16 +4321,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B231" t="str">
-        <v>Marca texto diferentes colores (1 para entregar)</v>
+        <v>Bolígrafo tinta roja (1 para entregar)</v>
       </c>
       <c r="C231">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D231" t="str">
-        <v>Marcatextos · 1 para entregar</v>
+        <v>Bolígrafo de tinta roja · 1 para entregar</v>
       </c>
       <c r="E231">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="232">
@@ -4338,16 +4338,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B232" t="str">
-        <v>Bolígrafo tinta negra (1 para entregar)</v>
+        <v>Jabón líquido para manos</v>
       </c>
       <c r="C232">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D232" t="str">
-        <v>Bolígrafo de tinta negra · 1 para entregar</v>
+        <v>Jabón líquido para manos 225 ml</v>
       </c>
       <c r="E232">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="233">
@@ -4355,16 +4355,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B233" t="str">
-        <v>Bolígrafo tinta azul (1 para entregar)</v>
+        <v>Paquete de conos para toma agua</v>
       </c>
       <c r="C233">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="D233" t="str">
-        <v>Bolígrafo de tinta azul · 1 para entregar</v>
+        <v>Paquete de conos para tomar agua</v>
       </c>
       <c r="E233">
-        <v>10</v>
+        <v>125</v>
       </c>
     </row>
     <row r="234">
@@ -4372,16 +4372,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B234" t="str">
-        <v>Bolígrafo tinta roja (1 para entregar)</v>
+        <v>Hojas de foami</v>
       </c>
       <c r="C234">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D234" t="str">
-        <v>Bolígrafo de tinta roja · 1 para entregar</v>
+        <v>Hoja de foami tamaño carta · Diferentes colores</v>
       </c>
       <c r="E234">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="235">
@@ -4389,16 +4389,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B235" t="str">
-        <v>Jabón líquido para manos</v>
+        <v>Hojas de foami diamantado</v>
       </c>
       <c r="C235">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="D235" t="str">
-        <v>Jabón líquido para manos 225 ml</v>
+        <v>Hoja de foami diamantado</v>
       </c>
       <c r="E235">
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="236">
@@ -4406,16 +4406,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B236" t="str">
-        <v>Paquete de conos para toma agua</v>
+        <v>Paquetes de sanitas</v>
       </c>
       <c r="C236">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="D236" t="str">
-        <v>Paquete de conos para tomar agua</v>
+        <v>Paquete de Sanitas</v>
       </c>
       <c r="E236">
-        <v>125</v>
+        <v>50</v>
       </c>
     </row>
     <row r="237">
@@ -4423,16 +4423,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B237" t="str">
-        <v>Hojas de foami</v>
+        <v>Silicón frío de 100ml</v>
       </c>
       <c r="C237">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="D237" t="str">
-        <v>Hoja de foami tamaño carta · Diferentes colores</v>
+        <v>Silicón frío 100 ml</v>
       </c>
       <c r="E237">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="238">
@@ -4440,16 +4440,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B238" t="str">
-        <v>Hojas de foami diamantado</v>
+        <v>Paquete de 50 protectores de hojas</v>
       </c>
       <c r="C238">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D238" t="str">
-        <v>Hoja de foami diamantado</v>
+        <v>Paquete de 50 protectores de hojas para carpeta</v>
       </c>
       <c r="E238">
-        <v>15</v>
+        <v>120</v>
       </c>
     </row>
     <row r="239">
@@ -4457,16 +4457,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B239" t="str">
-        <v>Paquetes de sanitas</v>
+        <v>Sobres de plástico rígido</v>
       </c>
       <c r="C239">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D239" t="str">
-        <v>Paquete de Sanitas</v>
+        <v>Sobre de plástico rígido</v>
       </c>
       <c r="E239">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="240">
@@ -4474,16 +4474,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B240" t="str">
-        <v>Silicón frío de 100ml</v>
+        <v>Pliego de papel américa colo amarillo</v>
       </c>
       <c r="C240">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D240" t="str">
-        <v>Silicón frío 100 ml</v>
+        <v>Pliego de papel américa amarillo</v>
       </c>
       <c r="E240">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="241">
@@ -4491,16 +4491,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B241" t="str">
-        <v>Paquete de 50 protectores de hojas</v>
+        <v>Pliegos de papel lustre (color a elegir)</v>
       </c>
       <c r="C241">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="D241" t="str">
-        <v>Paquete de 50 protectores de hojas para carpeta</v>
+        <v>Pliego de papel lustre · Color a elegir</v>
       </c>
       <c r="E241">
-        <v>120</v>
+        <v>15</v>
       </c>
     </row>
     <row r="242">
@@ -4508,16 +4508,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B242" t="str">
-        <v>Sobres de plástico rígido</v>
+        <v>Pliegos de papel Kraft</v>
       </c>
       <c r="C242">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="D242" t="str">
-        <v>Sobre de plástico rígido</v>
+        <v>Pliego de papel kraft</v>
       </c>
       <c r="E242">
-        <v>45</v>
+        <v>15</v>
       </c>
     </row>
     <row r="243">
@@ -4525,16 +4525,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B243" t="str">
-        <v>Pliego de papel américa colo amarillo</v>
+        <v>Masking tape</v>
       </c>
       <c r="C243">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D243" t="str">
-        <v>Pliego de papel américa amarillo</v>
+        <v>Cinta masking tape</v>
       </c>
       <c r="E243">
-        <v>30</v>
+        <v>45</v>
       </c>
     </row>
     <row r="244">
@@ -4542,16 +4542,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B244" t="str">
-        <v>Pliegos de papel lustre (color a elegir)</v>
+        <v>Fólders tamaña carta</v>
       </c>
       <c r="C244">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D244" t="str">
-        <v>Pliego de papel lustre · Color a elegir</v>
+        <v>Fólder tamaño carta beige</v>
       </c>
       <c r="E244">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="245">
@@ -4559,16 +4559,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B245" t="str">
-        <v>Pliegos de papel Kraft</v>
+        <v>Plumón para pizarrón blanco negro, rojo, verde y azul</v>
       </c>
       <c r="C245">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D245" t="str">
-        <v>Pliego de papel kraft</v>
+        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
       </c>
       <c r="E245">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="246">
@@ -4576,16 +4576,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B246" t="str">
-        <v>Masking tape</v>
+        <v>Diccionario escolar de la Lengua Española</v>
       </c>
       <c r="C246">
-        <v>45</v>
+        <v>182</v>
       </c>
       <c r="D246" t="str">
-        <v>Cinta masking tape</v>
+        <v>Diccionario escolar de la lengua española Larousse</v>
       </c>
       <c r="E246">
-        <v>45</v>
+        <v>182</v>
       </c>
     </row>
     <row r="247">
@@ -4593,16 +4593,16 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B247" t="str">
-        <v>Fólders tamaña carta</v>
+        <v>Get Involved! A1+ Student´s book (básico) ISBN: 9781380068750</v>
       </c>
       <c r="C247">
-        <v>7</v>
+        <v>1040</v>
       </c>
       <c r="D247" t="str">
-        <v>Fólder tamaño carta beige</v>
+        <v>Get Involved! A1+ Student's book ISBN: 9781380068750</v>
       </c>
       <c r="E247">
-        <v>7</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="248">
@@ -4610,67 +4610,67 @@
         <v>2do SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B248" t="str">
-        <v>Plumón para pizarrón blanco negro, rojo, verde y azul</v>
+        <v>Get Involved! B1 Student´s book (avanzado) ISBN: 9781380068873</v>
       </c>
       <c r="C248">
-        <v>35</v>
+        <v>1040</v>
       </c>
       <c r="D248" t="str">
-        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
+        <v>Get Involved! B1 Student's book ISBN: 9781380068873</v>
       </c>
       <c r="E248">
-        <v>35</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>2do SECUNDARIA VESPERTINO</v>
+        <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B249" t="str">
-        <v>Diccionario escolar de la Lengua Española</v>
+        <v>Cuadernos profesional cuadro chico 100. (Español, Inglés (forrado color verde), Química, Historia (2).</v>
       </c>
       <c r="C249">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="D249" t="str">
-        <v>Diccionario escolar de la lengua española Larousse</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Español, Inglés (forrado color verde), Química, Historia (2)</v>
       </c>
       <c r="E249">
-        <v>182</v>
+        <v>150</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>2do SECUNDARIA VESPERTINO</v>
+        <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B250" t="str">
-        <v>Get Involved! A1+ Student´s book (básico) ISBN: 9781380068750</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas Matemáticas</v>
       </c>
       <c r="C250">
-        <v>1040</v>
+        <v>150</v>
       </c>
       <c r="D250" t="str">
-        <v>Get Involved! A1+ Student's book ISBN: 9781380068750</v>
+        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
       </c>
       <c r="E250">
-        <v>1040</v>
+        <v>150</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>2do SECUNDARIA VESPERTINO</v>
+        <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B251" t="str">
-        <v>Get Involved! B1 Student´s book (avanzado) ISBN: 9781380068873</v>
+        <v>Bata blanca de algodón (bordada)</v>
       </c>
       <c r="C251">
-        <v>1040</v>
+        <v>300</v>
       </c>
       <c r="D251" t="str">
-        <v>Get Involved! B1 Student's book ISBN: 9781380068873</v>
+        <v>Bata blanca de algodón · Bordada</v>
       </c>
       <c r="E251">
-        <v>1040</v>
+        <v>300</v>
       </c>
     </row>
     <row r="252">
@@ -4678,16 +4678,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B252" t="str">
-        <v>Cuadernos profesional cuadro chico 100. (Español, Inglés (forrado color verde), Química, Historia (2).</v>
+        <v>Gomas (1 se entrega en la escuela)</v>
       </c>
       <c r="C252">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="D252" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Español, Inglés (forrado color verde), Química, Historia (2</v>
+        <v>Goma de migajón · 1 se entrega en la escuela</v>
       </c>
       <c r="E252">
-        <v>150</v>
+        <v>10</v>
       </c>
     </row>
     <row r="253">
@@ -4695,16 +4695,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B253" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas Matemáticas</v>
+        <v>Lápiz Mirado No. 2 (1 para entregar)</v>
       </c>
       <c r="C253">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="D253" t="str">
-        <v>Cuaderno profesional cuadro chico 100 hojas · Matemáticas</v>
+        <v>Lápiz No. 2 · 1 para entregar</v>
       </c>
       <c r="E253">
-        <v>150</v>
+        <v>10</v>
       </c>
     </row>
     <row r="254">
@@ -4712,16 +4712,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B254" t="str">
-        <v>Bata blanca de algodón (bordada)</v>
+        <v>Lápiz adhesivo (1 para entregar)</v>
       </c>
       <c r="C254">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="D254" t="str">
-        <v>Bata blanca de algodón · Bordada</v>
+        <v>Lápiz adhesivo tipo Pritt 22 g · 1 para entregar</v>
       </c>
       <c r="E254">
-        <v>300</v>
+        <v>40</v>
       </c>
     </row>
     <row r="255">
@@ -4729,16 +4729,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B255" t="str">
-        <v>Gomas (1 se entrega en la escuela)</v>
+        <v>Marcatexto diferente color (1 para entregar)</v>
       </c>
       <c r="C255">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D255" t="str">
-        <v>Goma de migajón · 1 se entrega en la escuela</v>
+        <v>Marcatextos · 1 para entregar</v>
       </c>
       <c r="E255">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="256">
@@ -4746,13 +4746,13 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B256" t="str">
-        <v>Lápiz Mirado No. 2 (1 para entregar)</v>
+        <v>Bolígrafo de tinta roja (1 para entregar)</v>
       </c>
       <c r="C256">
         <v>10</v>
       </c>
       <c r="D256" t="str">
-        <v>Lápiz No. 2 · 1 para entregar</v>
+        <v>Bolígrafo de tinta roja · 1 para entregar</v>
       </c>
       <c r="E256">
         <v>10</v>
@@ -4763,16 +4763,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B257" t="str">
-        <v>Lápiz adhesivo (1 para entregar)</v>
+        <v>Bolígrafo de tinta negra (1 para entregar)</v>
       </c>
       <c r="C257">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D257" t="str">
-        <v>Lápiz adhesivo tipo Pritt 22 g · 1 para entregar</v>
+        <v>Bolígrafo de tinta negra · 1 para entregar</v>
       </c>
       <c r="E257">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="258">
@@ -4780,16 +4780,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B258" t="str">
-        <v>Marcatexto diferente color (1 para entregar)</v>
+        <v>Bolígrafo de tinta azul (1 para entregar)</v>
       </c>
       <c r="C258">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="D258" t="str">
-        <v>Marcatextos · 1 para entregar</v>
+        <v>Bolígrafo de tinta azul · 1 para entregar</v>
       </c>
       <c r="E258">
-        <v>35</v>
+        <v>10</v>
       </c>
     </row>
     <row r="259">
@@ -4797,16 +4797,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B259" t="str">
-        <v>Bolígrafo de tinta roja (1 para entregar)</v>
+        <v>Tabla periódica actualizada</v>
       </c>
       <c r="C259">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D259" t="str">
-        <v>Bolígrafo de tinta roja · 1 para entregar</v>
+        <v>Tabla periódica actualizada Ed. Patria</v>
       </c>
       <c r="E259">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="260">
@@ -4814,16 +4814,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B260" t="str">
-        <v>Bolígrafo de tinta negra (1 para entregar)</v>
+        <v>Tijeras punta roma</v>
       </c>
       <c r="C260">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D260" t="str">
-        <v>Bolígrafo de tinta negra · 1 para entregar</v>
+        <v>Tijeras de punta roma</v>
       </c>
       <c r="E260">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="261">
@@ -4831,16 +4831,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B261" t="str">
-        <v>Bolígrafo de tinta azul (1 para entregar)</v>
+        <v>Jabón líquido para manos</v>
       </c>
       <c r="C261">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D261" t="str">
-        <v>Bolígrafo de tinta azul · 1 para entregar</v>
+        <v>Jabón líquido para manos 225 ml</v>
       </c>
       <c r="E261">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="262">
@@ -4848,16 +4848,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B262" t="str">
-        <v>Tabla periódica actualizada</v>
+        <v>Paquete de conos para toma agua</v>
       </c>
       <c r="C262">
-        <v>20</v>
+        <v>125</v>
       </c>
       <c r="D262" t="str">
-        <v>Tabla periódica actualizada Ed. Patria</v>
+        <v>Paquete de conos para tomar agua</v>
       </c>
       <c r="E262">
-        <v>20</v>
+        <v>125</v>
       </c>
     </row>
     <row r="263">
@@ -4865,16 +4865,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B263" t="str">
-        <v>Tijeras punta roma</v>
+        <v>Hojas de foami</v>
       </c>
       <c r="C263">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="D263" t="str">
-        <v>Tijeras de punta roma</v>
+        <v>Hoja de foami tamaño carta · Diferentes colores</v>
       </c>
       <c r="E263">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="264">
@@ -4882,16 +4882,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B264" t="str">
-        <v>Jabón líquido para manos</v>
+        <v>Hojas de foami diamantado</v>
       </c>
       <c r="C264">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="D264" t="str">
-        <v>Jabón líquido para manos 225 ml</v>
+        <v>Hoja de foami diamantado</v>
       </c>
       <c r="E264">
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="265">
@@ -4899,16 +4899,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B265" t="str">
-        <v>Paquete de conos para toma agua</v>
+        <v>Paquetes de sanitas</v>
       </c>
       <c r="C265">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="D265" t="str">
-        <v>Paquete de conos para tomar agua</v>
+        <v>Paquete de Sanitas</v>
       </c>
       <c r="E265">
-        <v>125</v>
+        <v>50</v>
       </c>
     </row>
     <row r="266">
@@ -4916,16 +4916,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B266" t="str">
-        <v>Hojas de foami</v>
+        <v>Silicón frío de 100ml</v>
       </c>
       <c r="C266">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="D266" t="str">
-        <v>Hoja de foami tamaño carta · Diferentes colores</v>
+        <v>Silicón frío 100 ml</v>
       </c>
       <c r="E266">
-        <v>5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="267">
@@ -4933,16 +4933,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B267" t="str">
-        <v>Hojas de foami diamantado</v>
+        <v>Paquete de 50 protectores de hojas</v>
       </c>
       <c r="C267">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D267" t="str">
-        <v>Hoja de foami diamantado</v>
+        <v>Paquete de 50 protectores de hojas para carpeta</v>
       </c>
       <c r="E267">
-        <v>15</v>
+        <v>120</v>
       </c>
     </row>
     <row r="268">
@@ -4950,16 +4950,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B268" t="str">
-        <v>Paquetes de sanitas</v>
+        <v>Sobres de plástico rígido</v>
       </c>
       <c r="C268">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D268" t="str">
-        <v>Paquete de Sanitas</v>
+        <v>Sobre de plástico rígido</v>
       </c>
       <c r="E268">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="269">
@@ -4967,16 +4967,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B269" t="str">
-        <v>Silicón frío de 100ml</v>
+        <v>Pliego de papel américa colo amarillo</v>
       </c>
       <c r="C269">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D269" t="str">
-        <v>Silicón frío 100 ml</v>
+        <v>Pliego de papel américa amarillo</v>
       </c>
       <c r="E269">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="270">
@@ -4984,16 +4984,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B270" t="str">
-        <v>Paquete de 50 protectores de hojas</v>
+        <v>Pliegos de papel lustre (color a elegir)</v>
       </c>
       <c r="C270">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="D270" t="str">
-        <v>Paquete de 50 protectores de hojas para carpeta</v>
+        <v>Pliego de papel lustre · Color a elegir</v>
       </c>
       <c r="E270">
-        <v>120</v>
+        <v>15</v>
       </c>
     </row>
     <row r="271">
@@ -5001,16 +5001,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B271" t="str">
-        <v>Sobres de plástico rígido</v>
+        <v>Pliegos de papel Kraft</v>
       </c>
       <c r="C271">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="D271" t="str">
-        <v>Sobre de plástico rígido</v>
+        <v>Pliego de papel kraft</v>
       </c>
       <c r="E271">
-        <v>45</v>
+        <v>15</v>
       </c>
     </row>
     <row r="272">
@@ -5018,16 +5018,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B272" t="str">
-        <v>Pliego de papel américa colo amarillo</v>
+        <v>Masking tape</v>
       </c>
       <c r="C272">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D272" t="str">
-        <v>Pliego de papel américa amarillo</v>
+        <v>Cinta masking tape</v>
       </c>
       <c r="E272">
-        <v>30</v>
+        <v>45</v>
       </c>
     </row>
     <row r="273">
@@ -5035,16 +5035,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B273" t="str">
-        <v>Pliegos de papel lustre (color a elegir)</v>
+        <v>Plumón para pizarrón blanco negro, rojo, verde y azul</v>
       </c>
       <c r="C273">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D273" t="str">
-        <v>Pliego de papel lustre · Color a elegir</v>
+        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
       </c>
       <c r="E273">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="274">
@@ -5052,16 +5052,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B274" t="str">
-        <v>Pliegos de papel Kraft</v>
+        <v>Diccionario escolar de la Lengua Española</v>
       </c>
       <c r="C274">
-        <v>15</v>
+        <v>182</v>
       </c>
       <c r="D274" t="str">
-        <v>Pliego de papel kraft</v>
+        <v>Diccionario escolar de la lengua española Larousse</v>
       </c>
       <c r="E274">
-        <v>15</v>
+        <v>182</v>
       </c>
     </row>
     <row r="275">
@@ -5069,16 +5069,16 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B275" t="str">
-        <v>Masking tape</v>
+        <v>Get Involved! A1+ Student´s book (básico) ISBN: 9781380068750</v>
       </c>
       <c r="C275">
-        <v>45</v>
+        <v>1040</v>
       </c>
       <c r="D275" t="str">
-        <v>Cinta masking tape</v>
+        <v>Get Involved! A1+ Student's book ISBN: 9781380068750</v>
       </c>
       <c r="E275">
-        <v>45</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="276">
@@ -5086,72 +5086,21 @@
         <v>3ro SECUNDARIA VESPERTINO</v>
       </c>
       <c r="B276" t="str">
-        <v>Plumón para pizarrón blanco negro, rojo, verde y azul</v>
+        <v>Get Involved! B1 Student´s book (avanzado) ISBN: 9781380068873</v>
       </c>
       <c r="C276">
-        <v>35</v>
+        <v>1040</v>
       </c>
       <c r="D276" t="str">
-        <v>Plumón para pizarrón blanco · Negro, rojo, verde y azul</v>
+        <v>Get Involved! B1 Student's book ISBN: 9781380068873</v>
       </c>
       <c r="E276">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="str">
-        <v>3ro SECUNDARIA VESPERTINO</v>
-      </c>
-      <c r="B277" t="str">
-        <v>Diccionario escolar de la Lengua Española</v>
-      </c>
-      <c r="C277">
-        <v>182</v>
-      </c>
-      <c r="D277" t="str">
-        <v>Diccionario escolar de la lengua española Larousse</v>
-      </c>
-      <c r="E277">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="str">
-        <v>3ro SECUNDARIA VESPERTINO</v>
-      </c>
-      <c r="B278" t="str">
-        <v>Get Involved! A1+ Student´s book (básico) ISBN: 9781380068750</v>
-      </c>
-      <c r="C278">
-        <v>1040</v>
-      </c>
-      <c r="D278" t="str">
-        <v>Get Involved! A1+ Student's book ISBN: 9781380068750</v>
-      </c>
-      <c r="E278">
-        <v>1040</v>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="str">
-        <v>3ro SECUNDARIA VESPERTINO</v>
-      </c>
-      <c r="B279" t="str">
-        <v>Get Involved! B1 Student´s book (avanzado) ISBN: 9781380068873</v>
-      </c>
-      <c r="C279">
-        <v>1040</v>
-      </c>
-      <c r="D279" t="str">
-        <v>Get Involved! B1 Student's book ISBN: 9781380068873</v>
-      </c>
-      <c r="E279">
         <v>1040</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E279"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E276"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>